<commit_message>
I cooked up some deadly spells analysis stuff
</commit_message>
<xml_diff>
--- a/final_output/mythicplus_tww.xlsx
+++ b/final_output/mythicplus_tww.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="262" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="164">
   <si>
     <t>Dungeon</t>
   </si>
@@ -45,244 +45,469 @@
     <t>Success</t>
   </si>
   <si>
-    <t>Save CC'd Ally</t>
-  </si>
-  <si>
-    <t>Overgrowth</t>
-  </si>
-  <si>
     <t>Defensive</t>
   </si>
   <si>
     <t>Furious Thrashing</t>
   </si>
   <si>
-    <t>Sidestep</t>
+    <t>1st boss</t>
+  </si>
+  <si>
+    <t>Swirls</t>
+  </si>
+  <si>
+    <t>Force Compliance</t>
+  </si>
+  <si>
+    <t>Fear</t>
+  </si>
+  <si>
+    <t>Repulsive Visage</t>
+  </si>
+  <si>
+    <t>Channel</t>
+  </si>
+  <si>
+    <t>2nd trash</t>
+  </si>
+  <si>
+    <t>Tongue Lashing</t>
+  </si>
+  <si>
+    <t>Radiant Breath</t>
+  </si>
+  <si>
+    <t>Poisonous Discharge</t>
+  </si>
+  <si>
+    <t>Pool of Radiance</t>
+  </si>
+  <si>
+    <t>Interrupt</t>
+  </si>
+  <si>
+    <t>Bramblethorn Coat</t>
+  </si>
+  <si>
+    <t>2nd boss</t>
+  </si>
+  <si>
+    <t>Dodge</t>
+  </si>
+  <si>
+    <t>CC Add</t>
+  </si>
+  <si>
+    <t>Freeze Tag</t>
+  </si>
+  <si>
+    <t>Patty Cake</t>
+  </si>
+  <si>
+    <t>Intermission</t>
+  </si>
+  <si>
+    <t>Guessing Game</t>
+  </si>
+  <si>
+    <t>3rd trash</t>
+  </si>
+  <si>
+    <t>3rd boss</t>
+  </si>
+  <si>
+    <t>Spread</t>
+  </si>
+  <si>
+    <t>Adds</t>
+  </si>
+  <si>
+    <t>The Necrotic Wake</t>
+  </si>
+  <si>
+    <t>Carrion Eruption</t>
+  </si>
+  <si>
+    <t>Rasping Scream</t>
+  </si>
+  <si>
+    <t>Gruesome Cleave</t>
+  </si>
+  <si>
+    <t>Dark Shroud</t>
+  </si>
+  <si>
+    <t>Move Out</t>
+  </si>
+  <si>
+    <t>Reaping Winds</t>
+  </si>
+  <si>
+    <t>Frigid Spikes</t>
+  </si>
+  <si>
+    <t>Spinning Frontal</t>
+  </si>
+  <si>
+    <t>Necrotic Breath</t>
+  </si>
+  <si>
+    <t>Goresplatter</t>
+  </si>
+  <si>
+    <t>Gut Slice</t>
+  </si>
+  <si>
+    <t>Meat Hook</t>
+  </si>
+  <si>
+    <t>4th boss</t>
+  </si>
+  <si>
+    <t>Comet Storm</t>
+  </si>
+  <si>
+    <t>ZoneID</t>
+  </si>
+  <si>
+    <t>Roles</t>
+  </si>
+  <si>
+    <t>All</t>
+  </si>
+  <si>
+    <t>Tank</t>
+  </si>
+  <si>
+    <t>SpellID</t>
+  </si>
+  <si>
+    <t>IconID</t>
+  </si>
+  <si>
+    <t>AbilityName</t>
+  </si>
+  <si>
+    <t>Bewildering Pollen</t>
+  </si>
+  <si>
+    <t>Frozen Binds</t>
+  </si>
+  <si>
+    <t>Grim Batol</t>
+  </si>
+  <si>
+    <t>Umbral Wind</t>
+  </si>
+  <si>
+    <t>Molten Mace</t>
+  </si>
+  <si>
+    <t>Kite Boss</t>
+  </si>
+  <si>
+    <t>Fiery Cleave</t>
+  </si>
+  <si>
+    <t>Ascension</t>
+  </si>
+  <si>
+    <t>Twilight Buffet</t>
+  </si>
+  <si>
+    <t>Knockback</t>
+  </si>
+  <si>
+    <t>Invocation of Shadowflame</t>
+  </si>
+  <si>
+    <t>Shadow Gale</t>
+  </si>
+  <si>
+    <t>Void Infusion</t>
+  </si>
+  <si>
+    <t>Coalescing Poison</t>
+  </si>
+  <si>
+    <t>Purge Massroot</t>
+  </si>
+  <si>
+    <t>Stop the Worm</t>
+  </si>
+  <si>
+    <t>Purge Miniboss</t>
+  </si>
+  <si>
+    <t>Big Defensive</t>
+  </si>
+  <si>
+    <t>Find Safespot</t>
+  </si>
+  <si>
+    <t>Move Miniboss</t>
+  </si>
+  <si>
+    <t>Frontal on me</t>
+  </si>
+  <si>
+    <t>Dodge Frontal</t>
+  </si>
+  <si>
+    <t>Ara-Kara, Echoes</t>
+  </si>
+  <si>
+    <t>Horrifying Shrill</t>
+  </si>
+  <si>
+    <t>Gossamer Onslaught</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alerting Shrill </t>
+  </si>
+  <si>
+    <t>Alarm went off</t>
+  </si>
+  <si>
+    <t>Alarm Shrill</t>
+  </si>
+  <si>
+    <t>Slam</t>
+  </si>
+  <si>
+    <t>Massive Slam</t>
+  </si>
+  <si>
+    <t>Venom Volley</t>
+  </si>
+  <si>
+    <t>Soak Puddle</t>
+  </si>
+  <si>
+    <t>Hide soon</t>
+  </si>
+  <si>
+    <t>Cosmic Singularity</t>
+  </si>
+  <si>
+    <t>Bait Swirls</t>
+  </si>
+  <si>
+    <t>City of Threads</t>
+  </si>
+  <si>
+    <t>Vociferous Indoctrination</t>
+  </si>
+  <si>
+    <t>Shadows of Doubt</t>
+  </si>
+  <si>
+    <t>Orbs</t>
+  </si>
+  <si>
+    <t>Gossamer Barrage</t>
+  </si>
+  <si>
+    <t>Synergic Step</t>
+  </si>
+  <si>
+    <t>Ice Sickles</t>
+  </si>
+  <si>
+    <t>Venomous Spray</t>
+  </si>
+  <si>
+    <t>Stack</t>
+  </si>
+  <si>
+    <t>Umbral Weave</t>
+  </si>
+  <si>
+    <t>4th trash</t>
+  </si>
+  <si>
+    <t>Dark Barrage</t>
+  </si>
+  <si>
+    <t>Tremor Slam</t>
+  </si>
+  <si>
+    <t>Perfume Toss</t>
+  </si>
+  <si>
+    <t>Dodge Ball (!)</t>
+  </si>
+  <si>
+    <t>Dodge Balls</t>
+  </si>
+  <si>
+    <t>Energy</t>
+  </si>
+  <si>
+    <t>Blood Surge</t>
+  </si>
+  <si>
+    <t>Viscous Darkness</t>
+  </si>
+  <si>
+    <t>Shifting Anomalies 23&amp;24</t>
+  </si>
+  <si>
+    <t>Shifting Anomalies 47&amp;48</t>
+  </si>
+  <si>
+    <t>Shifting Anomalies 65&amp;66</t>
+  </si>
+  <si>
+    <t>Shifting Anomalies 87&amp;88</t>
+  </si>
+  <si>
+    <t>Cosmic Singularity 84&amp;85</t>
+  </si>
+  <si>
+    <t>Dawnbreaker</t>
+  </si>
+  <si>
+    <t>Darkness Comes</t>
+  </si>
+  <si>
+    <t>Fly Away</t>
+  </si>
+  <si>
+    <t>Collapsing Night</t>
+  </si>
+  <si>
+    <t>Terrifying Slam</t>
+  </si>
+  <si>
+    <t>Dark Orb</t>
+  </si>
+  <si>
+    <t>Shadowy Decay</t>
+  </si>
+  <si>
+    <t>No one in Range</t>
+  </si>
+  <si>
+    <t>Tacky Burst</t>
+  </si>
+  <si>
+    <t>Bait Orb</t>
+  </si>
+  <si>
+    <t>The Stonevaults</t>
+  </si>
+  <si>
+    <t>Howling Fear</t>
+  </si>
+  <si>
+    <t>Earth Shattere</t>
+  </si>
+  <si>
+    <t>Scrap Song</t>
+  </si>
+  <si>
+    <t>Exhaust Vents</t>
+  </si>
+  <si>
+    <t>Blazing Crescendo</t>
+  </si>
+  <si>
+    <t>Crystal Salvo</t>
+  </si>
+  <si>
+    <t>Void Outburst</t>
+  </si>
+  <si>
+    <t>Void Discharge</t>
+  </si>
+  <si>
+    <t>Soak Orbs</t>
+  </si>
+  <si>
+    <t>Fortified Shell</t>
+  </si>
+  <si>
+    <t>Bait</t>
+  </si>
+  <si>
+    <t>Earth Burst Totem</t>
+  </si>
+  <si>
+    <t>Totem</t>
+  </si>
+  <si>
+    <t>Smash Rock</t>
+  </si>
+  <si>
+    <t>Void Corruption</t>
+  </si>
+  <si>
+    <t>Debuffs</t>
+  </si>
+  <si>
+    <t>Flame Cannon</t>
+  </si>
+  <si>
+    <t>Embrace Darkness</t>
+  </si>
+  <si>
+    <t>Boss Immunity</t>
   </si>
   <si>
     <t>Bramble Burst</t>
   </si>
   <si>
-    <t>1st boss</t>
-  </si>
-  <si>
-    <t>Swirls</t>
-  </si>
-  <si>
-    <t>Force Compliance</t>
-  </si>
-  <si>
-    <t>Fear</t>
-  </si>
-  <si>
-    <t>Repulsive Visage</t>
-  </si>
-  <si>
-    <t>Channel</t>
-  </si>
-  <si>
-    <t>2nd trash</t>
-  </si>
-  <si>
-    <t>Tongue Lashing</t>
-  </si>
-  <si>
-    <t>Radiant Breath</t>
-  </si>
-  <si>
-    <t>Poisonous Discharge</t>
-  </si>
-  <si>
-    <t>Move Enemy</t>
-  </si>
-  <si>
-    <t>Pool of Radiance</t>
-  </si>
-  <si>
-    <t>Interrupt</t>
-  </si>
-  <si>
-    <t>Bramblethorn Coat</t>
-  </si>
-  <si>
-    <t>2nd boss</t>
-  </si>
-  <si>
-    <t>Dodge</t>
-  </si>
-  <si>
-    <t>CC Add</t>
-  </si>
-  <si>
-    <t>Freeze Tag</t>
-  </si>
-  <si>
-    <t>Failed Kick</t>
-  </si>
-  <si>
-    <t>Patty Cake</t>
-  </si>
-  <si>
-    <t>Intermission</t>
-  </si>
-  <si>
-    <t>Guessing Game</t>
-  </si>
-  <si>
-    <t>3rd trash</t>
+    <t>Kick</t>
+  </si>
+  <si>
+    <t>Disorient on Tank</t>
+  </si>
+  <si>
+    <t>Healer</t>
   </si>
   <si>
     <t>Stimulate Resistance</t>
   </si>
   <si>
-    <t>3rd boss</t>
-  </si>
-  <si>
-    <t>Spread</t>
-  </si>
-  <si>
-    <t>Adds</t>
-  </si>
-  <si>
-    <t>The Necrotic Wake</t>
-  </si>
-  <si>
-    <t>Heaving Retch</t>
-  </si>
-  <si>
-    <t>Carrion Eruption</t>
-  </si>
-  <si>
-    <t>Rasping Scream</t>
-  </si>
-  <si>
-    <t>Gruesome Cleave</t>
-  </si>
-  <si>
-    <t>Dark Shroud</t>
-  </si>
-  <si>
-    <t>Move Out</t>
-  </si>
-  <si>
-    <t>Reaping Winds</t>
-  </si>
-  <si>
-    <t>Frigid Spikes</t>
-  </si>
-  <si>
-    <t>Spinning Frontal</t>
-  </si>
-  <si>
-    <t>Necrotic Breath</t>
-  </si>
-  <si>
-    <t>Goresplatter</t>
-  </si>
-  <si>
-    <t>Gut Slice</t>
-  </si>
-  <si>
-    <t>Hook boss</t>
-  </si>
-  <si>
-    <t>Meat Hook</t>
-  </si>
-  <si>
-    <t>4th boss</t>
-  </si>
-  <si>
-    <t>Comet Storm</t>
-  </si>
-  <si>
-    <t>ZoneID</t>
-  </si>
-  <si>
-    <t>Roles</t>
-  </si>
-  <si>
-    <t>All</t>
-  </si>
-  <si>
-    <t>Tank</t>
-  </si>
-  <si>
-    <t>SpellID</t>
-  </si>
-  <si>
-    <t>IconID</t>
-  </si>
-  <si>
-    <t>AbilityName</t>
-  </si>
-  <si>
-    <t>Bewildering Pollen</t>
-  </si>
-  <si>
-    <t>Frozen Binds</t>
-  </si>
-  <si>
-    <t>Grim Batol</t>
-  </si>
-  <si>
-    <t>Umbral Wind</t>
-  </si>
-  <si>
-    <t>Mass Tremor</t>
-  </si>
-  <si>
-    <t>Molten Mace</t>
-  </si>
-  <si>
-    <t>Kite Boss</t>
-  </si>
-  <si>
-    <t>Fiery Cleave</t>
-  </si>
-  <si>
-    <t>Ascension</t>
-  </si>
-  <si>
-    <t>Twilight Buffet</t>
-  </si>
-  <si>
-    <t>Knockback</t>
-  </si>
-  <si>
-    <t>Invocation of Shadowflame</t>
-  </si>
-  <si>
-    <t>Shadow Gale</t>
-  </si>
-  <si>
-    <t>Void Infusion</t>
-  </si>
-  <si>
-    <t>Player</t>
-  </si>
-  <si>
-    <t>Coalescing Poison</t>
-  </si>
-  <si>
     <t>Nova</t>
   </si>
   <si>
     <t>Acid Nova</t>
   </si>
   <si>
-    <t>Purge Massroot</t>
-  </si>
-  <si>
-    <t>Stop the Worm</t>
-  </si>
-  <si>
-    <t>Purge Miniboss</t>
-  </si>
-  <si>
-    <t>Big Defensive</t>
-  </si>
-  <si>
-    <t>Find Safespot</t>
+    <t>Hook Boss</t>
+  </si>
+  <si>
+    <t>Erupting Webs</t>
+  </si>
+  <si>
+    <t>Revolting Volley</t>
+  </si>
+  <si>
+    <t>Poison Dispel</t>
+  </si>
+  <si>
+    <t>Ravenous Swarm</t>
+  </si>
+  <si>
+    <t>Move Away</t>
+  </si>
+  <si>
+    <t>Dance</t>
+  </si>
+  <si>
+    <t>Avoid Me</t>
+  </si>
+  <si>
+    <t>Process of Elimination</t>
+  </si>
+  <si>
+    <t>Obsidian Beam</t>
+  </si>
+  <si>
+    <t>Spinning Beam</t>
   </si>
 </sst>
 </file>
@@ -343,7 +568,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -373,6 +598,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -667,7 +896,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J44"/>
+  <dimension ref="A1:J97"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.28515625" customWidth="1"/>
@@ -675,8 +904,8 @@
     <col min="3" max="3" width="10.140625" customWidth="1"/>
     <col min="4" max="4" width="7.85546875" customWidth="1"/>
     <col min="5" max="5" width="3.140625" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" customWidth="1"/>
-    <col min="7" max="7" width="21.85546875" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" customWidth="1"/>
+    <col min="7" max="7" width="25.42578125" customWidth="1"/>
     <col min="8" max="8" width="8.42578125" customWidth="1"/>
     <col min="9" max="9" width="8" customWidth="1"/>
     <col min="10" max="10" width="9.42578125" customWidth="1"/>
@@ -687,7 +916,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="10" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C1" s="10" t="s">
         <v>1</v>
@@ -702,16 +931,16 @@
         <v>4</v>
       </c>
       <c r="G1" s="10" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="H1" s="11" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="I1" s="11" t="s">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="J1" s="11" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -728,13 +957,13 @@
         <v>2</v>
       </c>
       <c r="E2" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>7</v>
+        <v>77</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>66</v>
+        <v>57</v>
       </c>
       <c r="H2" s="1">
         <v>321968</v>
@@ -743,7 +972,7 @@
         <v>-1</v>
       </c>
       <c r="J2" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -757,25 +986,25 @@
         <v>6</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E3" s="2">
         <v>0</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>10</v>
+        <v>146</v>
       </c>
       <c r="H3" s="1">
-        <v>322486</v>
+        <v>324923</v>
       </c>
       <c r="I3" s="1">
-        <v>959842</v>
+        <v>-1</v>
       </c>
       <c r="J3" t="s">
-        <v>80</v>
+        <v>52</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -795,19 +1024,19 @@
         <v>0</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="H4" s="1">
-        <v>324923</v>
+        <v>324909</v>
       </c>
       <c r="I4" s="1">
         <v>-1</v>
       </c>
       <c r="J4" t="s">
-        <v>61</v>
+        <v>149</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -817,8 +1046,8 @@
       <c r="B5" s="1">
         <v>13334</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>6</v>
+      <c r="C5" s="1" t="s">
+        <v>11</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>2</v>
@@ -827,19 +1056,19 @@
         <v>0</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H5" s="1">
-        <v>324909</v>
+        <v>323138</v>
       </c>
       <c r="I5" s="1">
         <v>-1</v>
       </c>
       <c r="J5" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="6" spans="1:10">
@@ -850,28 +1079,28 @@
         <v>13334</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E6" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>16</v>
+        <v>145</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>17</v>
+        <v>144</v>
       </c>
       <c r="H6" s="1">
-        <v>323138</v>
+        <v>323149</v>
       </c>
       <c r="I6" s="1">
         <v>-1</v>
       </c>
       <c r="J6" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -882,19 +1111,19 @@
         <v>13334</v>
       </c>
       <c r="C7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" s="2">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E7" s="2">
-        <v>0</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="H7" s="1">
         <v>328756</v>
@@ -903,7 +1132,7 @@
         <v>-1</v>
       </c>
       <c r="J7" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="8" spans="1:10">
@@ -914,19 +1143,19 @@
         <v>13334</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E8" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>7</v>
+        <v>78</v>
       </c>
       <c r="G8" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="H8">
         <v>340160</v>
@@ -935,7 +1164,7 @@
         <v>-1</v>
       </c>
       <c r="J8" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -946,19 +1175,19 @@
         <v>13334</v>
       </c>
       <c r="C9" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" s="2">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="G9" t="s">
         <v>21</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E9" s="2">
-        <v>0</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="G9" t="s">
-        <v>26</v>
       </c>
       <c r="H9">
         <v>340189</v>
@@ -967,7 +1196,7 @@
         <v>-1</v>
       </c>
       <c r="J9" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:10">
@@ -978,19 +1207,19 @@
         <v>13334</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E10" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>7</v>
+        <v>78</v>
       </c>
       <c r="G10" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="H10">
         <v>340300</v>
@@ -999,7 +1228,7 @@
         <v>-1</v>
       </c>
       <c r="J10" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -1010,19 +1239,19 @@
         <v>13334</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E11" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G11" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="H11">
         <v>340279</v>
@@ -1031,7 +1260,7 @@
         <v>-1</v>
       </c>
       <c r="J11" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -1042,28 +1271,28 @@
         <v>13334</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E12" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>84</v>
+        <v>71</v>
       </c>
       <c r="G12" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="H12">
         <v>324776</v>
       </c>
-      <c r="I12" s="4">
-        <v>-1</v>
+      <c r="I12">
+        <v>136006</v>
       </c>
       <c r="J12" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -1074,19 +1303,19 @@
         <v>13334</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E13" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="G13" s="4" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="H13" s="4">
         <v>341709</v>
@@ -1095,7 +1324,7 @@
         <v>-1</v>
       </c>
       <c r="J13" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:10">
@@ -1106,19 +1335,19 @@
         <v>13334</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>8</v>
       </c>
       <c r="E14" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>33</v>
+        <v>148</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="H14" s="1">
         <v>321828</v>
@@ -1127,7 +1356,7 @@
         <v>134470</v>
       </c>
       <c r="J14" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1137,29 +1366,29 @@
       <c r="B15" s="1">
         <v>13334</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" s="5" t="s">
+      <c r="C15" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E15" s="2">
         <v>0</v>
       </c>
-      <c r="F15" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="H15" s="4">
-        <v>336499</v>
+      <c r="F15" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="H15" s="1">
+        <v>321834</v>
       </c>
       <c r="I15" s="4">
         <v>-1</v>
       </c>
       <c r="J15" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -1169,29 +1398,29 @@
       <c r="B16" s="1">
         <v>13334</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="D16" s="2" t="s">
+      <c r="C16" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E16" s="2">
         <v>0</v>
       </c>
-      <c r="F16" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G16" t="s">
-        <v>38</v>
-      </c>
-      <c r="H16">
-        <v>326046</v>
+      <c r="F16" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H16" s="4">
+        <v>336499</v>
       </c>
       <c r="I16" s="4">
         <v>-1</v>
       </c>
       <c r="J16" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="17" spans="1:10">
@@ -1202,28 +1431,28 @@
         <v>13334</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D17" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E17" s="2">
         <v>0</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>82</v>
+        <v>147</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="H17">
-        <v>460092</v>
+        <v>150</v>
+      </c>
+      <c r="H17" s="4">
+        <v>326046</v>
       </c>
       <c r="I17" s="4">
         <v>-1</v>
       </c>
       <c r="J17" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:10">
@@ -1233,72 +1462,72 @@
       <c r="B18" s="1">
         <v>13334</v>
       </c>
-      <c r="C18" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D18" s="2" t="s">
+      <c r="C18" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="5" t="s">
         <v>2</v>
       </c>
       <c r="E18" s="2">
         <v>0</v>
       </c>
-      <c r="F18" s="3" t="s">
-        <v>48</v>
+      <c r="F18" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="H18">
+        <v>152</v>
+      </c>
+      <c r="H18" s="4">
+        <v>460092</v>
+      </c>
+      <c r="I18" s="4">
+        <v>-1</v>
+      </c>
+      <c r="J18" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="19" spans="1:10" s="9" customFormat="1" ht="15.75" thickBot="1">
+      <c r="A19" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="B19" s="6">
+        <v>13334</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D19" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="E19" s="8">
+        <v>0</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="H19" s="9">
         <v>463602</v>
       </c>
-      <c r="I18" s="4">
-        <v>-1</v>
-      </c>
-      <c r="J18" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="19" spans="1:10" s="14" customFormat="1">
-      <c r="A19" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="B19" s="1">
-        <v>12917</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E19" s="2">
-        <v>0</v>
-      </c>
-      <c r="F19" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="G19" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="H19" s="14">
-        <v>320596</v>
-      </c>
-      <c r="I19" s="4">
-        <v>-1</v>
-      </c>
-      <c r="J19" s="14" t="s">
-        <v>80</v>
+      <c r="I19" s="7">
+        <v>-1</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B20" s="1">
         <v>12917</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>2</v>
@@ -1307,10 +1536,10 @@
         <v>0</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>85</v>
+        <v>72</v>
       </c>
       <c r="G20" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="H20">
         <v>320631</v>
@@ -1319,18 +1548,18 @@
         <v>-1</v>
       </c>
       <c r="J20" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B21" s="1">
         <v>12917</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>8</v>
@@ -1339,10 +1568,10 @@
         <v>0</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="G21" t="s">
-        <v>44</v>
+        <v>36</v>
       </c>
       <c r="H21">
         <v>320631</v>
@@ -1351,18 +1580,18 @@
         <v>136030</v>
       </c>
       <c r="J21" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:10">
       <c r="A22" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B22" s="1">
         <v>12917</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>2</v>
@@ -1371,10 +1600,10 @@
         <v>0</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G22" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
       <c r="H22">
         <v>324293</v>
@@ -1383,18 +1612,18 @@
         <v>-1</v>
       </c>
       <c r="J22" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="23" spans="1:10">
       <c r="A23" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B23" s="1">
         <v>12917</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>2</v>
@@ -1406,7 +1635,7 @@
         <v>7</v>
       </c>
       <c r="G23" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="H23">
         <v>324323</v>
@@ -1415,18 +1644,18 @@
         <v>-1</v>
       </c>
       <c r="J23" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
     </row>
     <row r="24" spans="1:10">
       <c r="A24" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B24" s="1">
         <v>12917</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>2</v>
@@ -1435,10 +1664,10 @@
         <v>0</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G24" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H24">
         <v>335141</v>
@@ -1447,18 +1676,18 @@
         <v>2576096</v>
       </c>
       <c r="J24" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="25" spans="1:10">
       <c r="A25" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B25" s="1">
         <v>12917</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>8</v>
@@ -1467,10 +1696,10 @@
         <v>0</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="G25" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="H25">
         <v>335141</v>
@@ -1479,30 +1708,30 @@
         <v>-1</v>
       </c>
       <c r="J25" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="26" spans="1:10">
       <c r="A26" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B26" s="1">
         <v>12917</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E26" s="2">
         <v>0</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="G26" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="H26">
         <v>324372</v>
@@ -1511,18 +1740,18 @@
         <v>-1</v>
       </c>
       <c r="J26" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="27" spans="1:10">
       <c r="A27" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B27" s="1">
         <v>12917</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>2</v>
@@ -1531,10 +1760,10 @@
         <v>0</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G27" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="H27">
         <v>324387</v>
@@ -1543,18 +1772,18 @@
         <v>-1</v>
       </c>
       <c r="J27" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="28" spans="1:10">
       <c r="A28" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B28" s="1">
         <v>12917</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>2</v>
@@ -1563,10 +1792,10 @@
         <v>0</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="G28" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="H28">
         <v>333488</v>
@@ -1575,30 +1804,30 @@
         <v>-1</v>
       </c>
       <c r="J28" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="29" spans="1:10">
       <c r="A29" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B29" s="1">
         <v>12917</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E29" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="G29" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="H29">
         <v>338353</v>
@@ -1607,18 +1836,18 @@
         <v>-1</v>
       </c>
       <c r="J29" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="30" spans="1:10">
       <c r="A30" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B30" s="1">
         <v>12917</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>8</v>
@@ -1627,10 +1856,10 @@
         <v>0</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="G30" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="H30">
         <v>338353</v>
@@ -1639,18 +1868,18 @@
         <v>-1</v>
       </c>
       <c r="J30" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:10">
       <c r="A31" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B31" s="1">
         <v>12917</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="D31" s="2" t="s">
         <v>2</v>
@@ -1659,10 +1888,10 @@
         <v>0</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G31" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="H31">
         <v>333477</v>
@@ -1671,30 +1900,30 @@
         <v>-1</v>
       </c>
       <c r="J31" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="32" spans="1:10">
       <c r="A32" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B32" s="1">
         <v>12917</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E32" s="2">
         <v>0</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>55</v>
+        <v>153</v>
       </c>
       <c r="G32" t="s">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="H32">
         <v>322681</v>
@@ -1703,30 +1932,30 @@
         <v>-1</v>
       </c>
       <c r="J32" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="33" spans="1:10">
       <c r="A33" s="1" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B33" s="1">
         <v>12917</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D33" s="2" t="s">
         <v>2</v>
       </c>
       <c r="E33" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="G33" t="s">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="H33">
         <v>320772</v>
@@ -1735,30 +1964,30 @@
         <v>-1</v>
       </c>
       <c r="J33" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="34" spans="1:10" s="9" customFormat="1" ht="15.75" thickBot="1">
       <c r="A34" s="6" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B34" s="6">
         <v>12917</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="D34" s="8" t="s">
         <v>2</v>
       </c>
       <c r="E34" s="8">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="H34" s="9">
         <v>320788</v>
@@ -1767,12 +1996,12 @@
         <v>-1</v>
       </c>
       <c r="J34" s="9" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="35" spans="1:10">
       <c r="A35" s="4" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="C35" s="12" t="s">
         <v>6</v>
@@ -1780,208 +2009,1540 @@
       <c r="D35" s="12" t="s">
         <v>2</v>
       </c>
+      <c r="E35" s="12">
+        <v>1</v>
+      </c>
       <c r="F35" s="4" t="s">
-        <v>76</v>
+        <v>66</v>
       </c>
       <c r="G35" t="s">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="H35">
         <v>451939</v>
       </c>
+      <c r="I35" s="4">
+        <v>-1</v>
+      </c>
       <c r="J35" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="36" spans="1:10">
       <c r="A36" s="4" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="C36" s="12" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="D36" s="12" t="s">
         <v>2</v>
       </c>
+      <c r="E36" s="12">
+        <v>1</v>
+      </c>
       <c r="F36" s="4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="G36" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="H36">
-        <v>451871</v>
+        <v>447395</v>
+      </c>
+      <c r="I36" s="4">
+        <v>-1</v>
       </c>
       <c r="J36" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="37" spans="1:10">
       <c r="A37" s="4" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="C37" s="12" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D37" s="12" t="s">
         <v>2</v>
       </c>
+      <c r="E37" s="12">
+        <v>1</v>
+      </c>
       <c r="F37" s="4" t="s">
-        <v>30</v>
+        <v>62</v>
       </c>
       <c r="G37" t="s">
-        <v>73</v>
+        <v>61</v>
       </c>
       <c r="H37">
-        <v>447395</v>
+        <v>449687</v>
+      </c>
+      <c r="I37" s="4">
+        <v>-1</v>
       </c>
       <c r="J37" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="38" spans="1:10">
       <c r="A38" s="4" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="C38" s="12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D38" s="12" t="s">
         <v>2</v>
       </c>
+      <c r="E38" s="12">
+        <v>1</v>
+      </c>
       <c r="F38" s="4" t="s">
-        <v>72</v>
+        <v>9</v>
       </c>
       <c r="G38" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="H38">
-        <v>449687</v>
+        <v>451387</v>
+      </c>
+      <c r="I38" s="4">
+        <v>-1</v>
       </c>
       <c r="J38" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="39" spans="1:10">
       <c r="A39" s="4" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="D39" s="12" t="s">
         <v>2</v>
       </c>
+      <c r="E39" s="12">
+        <v>1</v>
+      </c>
       <c r="F39" s="4" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="G39" t="s">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="H39">
-        <v>451387</v>
+        <v>456751</v>
+      </c>
+      <c r="I39" s="4">
+        <v>-1</v>
       </c>
       <c r="J39" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="40" spans="1:10">
       <c r="A40" s="4" t="s">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D40" s="12" t="s">
         <v>2</v>
       </c>
+      <c r="E40" s="12">
+        <v>1</v>
+      </c>
       <c r="F40" s="4" t="s">
-        <v>76</v>
+        <v>34</v>
       </c>
       <c r="G40" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="H40">
-        <v>456751</v>
+        <v>448013</v>
+      </c>
+      <c r="I40" s="4">
+        <v>-1</v>
       </c>
       <c r="J40" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41" spans="1:10">
       <c r="A41" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D41" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E41" s="12">
+        <v>1</v>
+      </c>
+      <c r="F41" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="G41" t="s">
         <v>68</v>
       </c>
-      <c r="C41" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="D41" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="F41" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="G41" t="s">
-        <v>77</v>
-      </c>
       <c r="H41">
-        <v>448013</v>
+        <v>449939</v>
+      </c>
+      <c r="I41" s="4">
+        <v>-1</v>
       </c>
       <c r="J41" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10">
-      <c r="A42" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C42" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="D42" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="F42" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" s="9" customFormat="1" ht="15.75" thickBot="1">
+      <c r="A42" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C42" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="E42" s="9">
+        <v>1</v>
+      </c>
+      <c r="F42" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="G42" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="H42" s="9">
+        <v>450088</v>
+      </c>
+      <c r="I42" s="9">
+        <v>-1</v>
+      </c>
+      <c r="J42" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10">
+      <c r="A43" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D43" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E43" s="12">
+        <v>1</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G43" t="s">
+        <v>80</v>
+      </c>
+      <c r="H43">
+        <v>434802</v>
+      </c>
+      <c r="I43" s="4">
+        <v>-1</v>
+      </c>
+      <c r="J43" s="16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10">
+      <c r="A44" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D44" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E44" s="12">
+        <v>1</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="G44" t="s">
+        <v>81</v>
+      </c>
+      <c r="H44">
+        <v>438473</v>
+      </c>
+      <c r="I44" s="4">
+        <v>-1</v>
+      </c>
+      <c r="J44" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10">
+      <c r="A45" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D45" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G45" t="s">
+        <v>82</v>
+      </c>
+      <c r="H45">
+        <v>438476</v>
+      </c>
+      <c r="I45" s="4">
+        <v>-1</v>
+      </c>
+      <c r="J45" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10">
+      <c r="A46" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D46" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G46" t="s">
+        <v>84</v>
+      </c>
+      <c r="H46">
+        <v>432967</v>
+      </c>
+      <c r="I46">
+        <v>120855</v>
+      </c>
+      <c r="J46" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10">
+      <c r="A47" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D47" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G47" t="s">
+        <v>86</v>
+      </c>
+      <c r="H47">
+        <v>434252</v>
+      </c>
+      <c r="I47" s="4">
+        <v>-1</v>
+      </c>
+      <c r="J47" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10">
+      <c r="A48" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D48" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="G48" t="s">
+        <v>155</v>
+      </c>
+      <c r="H48">
+        <v>448248</v>
+      </c>
+      <c r="I48">
+        <v>5094557</v>
+      </c>
+      <c r="J48" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10">
+      <c r="A49" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D49" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>156</v>
+      </c>
+      <c r="G49" t="s">
+        <v>87</v>
+      </c>
+      <c r="H49">
+        <v>433841</v>
+      </c>
+      <c r="I49">
+        <v>132108</v>
+      </c>
+      <c r="J49" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10">
+      <c r="A50" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D50" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G50" t="s">
+        <v>154</v>
+      </c>
+      <c r="H50">
+        <v>433845</v>
+      </c>
+      <c r="I50">
+        <v>-1</v>
+      </c>
+      <c r="J50" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10">
+      <c r="A51" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D51" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F51" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G51" t="s">
+        <v>154</v>
+      </c>
+      <c r="H51">
+        <v>432130</v>
+      </c>
+      <c r="I51">
+        <v>-1</v>
+      </c>
+      <c r="J51" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10">
+      <c r="A52" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C52" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D52" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F52" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="G42" t="s">
-        <v>78</v>
-      </c>
-      <c r="H42">
-        <v>449939</v>
-      </c>
-      <c r="J42" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" s="9" customFormat="1" ht="15.75" thickBot="1">
-      <c r="A43" s="7" t="s">
-        <v>68</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>57</v>
-      </c>
-      <c r="D43" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="F43" s="7" t="s">
-        <v>41</v>
-      </c>
-      <c r="G43" s="9" t="s">
+      <c r="G52" t="s">
+        <v>90</v>
+      </c>
+      <c r="H52">
+        <v>432117</v>
+      </c>
+      <c r="I52">
+        <v>-1</v>
+      </c>
+      <c r="J52" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" s="9" customFormat="1" ht="15.75" thickBot="1">
+      <c r="A53" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="H43" s="9">
-        <v>450088</v>
-      </c>
-      <c r="J43" s="9" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10">
-      <c r="A44" s="4"/>
+      <c r="C53" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D53" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="F53" s="7" t="s">
+        <v>89</v>
+      </c>
+      <c r="G53" s="9" t="s">
+        <v>115</v>
+      </c>
+      <c r="H53" s="9">
+        <v>432117</v>
+      </c>
+      <c r="I53" s="9">
+        <v>4914670</v>
+      </c>
+      <c r="J53" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" s="14" customFormat="1">
+      <c r="A54" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D54" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F54" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G54" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="H54" s="14">
+        <v>443507</v>
+      </c>
+      <c r="I54" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J54" s="16" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" s="14" customFormat="1">
+      <c r="A55" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B55"/>
+      <c r="C55" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D55" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="E55"/>
+      <c r="F55" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G55" t="s">
+        <v>94</v>
+      </c>
+      <c r="H55">
+        <v>443436</v>
+      </c>
+      <c r="I55" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J55" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10">
+      <c r="A56" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D56" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G56" t="s">
+        <v>94</v>
+      </c>
+      <c r="H56">
+        <v>448560</v>
+      </c>
+      <c r="I56" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J56" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10">
+      <c r="A57" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D57" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>158</v>
+      </c>
+      <c r="G57" t="s">
+        <v>93</v>
+      </c>
+      <c r="H57">
+        <v>434829</v>
+      </c>
+      <c r="I57" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J57" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10">
+      <c r="A58" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C58" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D58" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G58" t="s">
+        <v>105</v>
+      </c>
+      <c r="H58">
+        <v>450784</v>
+      </c>
+      <c r="I58" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J58" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10">
+      <c r="A59" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D59" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G59" t="s">
+        <v>96</v>
+      </c>
+      <c r="H59">
+        <v>451423</v>
+      </c>
+      <c r="I59" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J59" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10">
+      <c r="A60" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C60" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D60" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="G60" t="s">
+        <v>97</v>
+      </c>
+      <c r="H60">
+        <v>441381</v>
+      </c>
+      <c r="I60" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J60" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10">
+      <c r="A61" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C61" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D61" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="G61" t="s">
+        <v>98</v>
+      </c>
+      <c r="H61">
+        <v>440218</v>
+      </c>
+      <c r="I61" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J61" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10">
+      <c r="A62" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C62" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D62" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G62" t="s">
+        <v>99</v>
+      </c>
+      <c r="H62">
+        <v>434137</v>
+      </c>
+      <c r="I62" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J62" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="63" spans="1:10">
+      <c r="A63" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C63" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D63" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F63" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G63" t="s">
+        <v>103</v>
+      </c>
+      <c r="H63">
+        <v>445813</v>
+      </c>
+      <c r="I63" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J63" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="64" spans="1:10">
+      <c r="A64" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C64" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D64" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G64" t="s">
+        <v>110</v>
+      </c>
+      <c r="H64">
+        <v>441289</v>
+      </c>
+      <c r="I64" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J64" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="65" spans="1:10">
+      <c r="A65" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C65" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D65" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G65" t="s">
+        <v>109</v>
+      </c>
+      <c r="H65">
+        <v>461880</v>
+      </c>
+      <c r="I65" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J65" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10">
+      <c r="A66" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C66" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="D66" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F66" t="s">
+        <v>100</v>
+      </c>
+      <c r="G66" t="s">
+        <v>101</v>
+      </c>
+      <c r="H66">
+        <v>446717</v>
+      </c>
+      <c r="I66" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J66" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10">
+      <c r="A67" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C67" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="D67" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G67" t="s">
+        <v>104</v>
+      </c>
+      <c r="H67">
+        <v>447271</v>
+      </c>
+      <c r="I67" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J67" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10">
+      <c r="A68" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C68" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D68" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="G68" t="s">
+        <v>101</v>
+      </c>
+      <c r="H68">
+        <v>438860</v>
+      </c>
+      <c r="I68" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J68" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="69" spans="1:10">
+      <c r="A69" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C69" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D69" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G69" t="s">
+        <v>161</v>
+      </c>
+      <c r="H69">
+        <v>439646</v>
+      </c>
+      <c r="I69" s="16">
+        <v>-1</v>
+      </c>
+      <c r="J69" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="70" spans="1:10">
+      <c r="A70" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C70" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D70" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="F70" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G70" t="s">
+        <v>111</v>
+      </c>
+      <c r="H70">
+        <v>439401</v>
+      </c>
+      <c r="I70">
+        <v>4914670</v>
+      </c>
+      <c r="J70" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="71" spans="1:10">
+      <c r="A71" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C71" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D71" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G71" t="s">
+        <v>112</v>
+      </c>
+      <c r="H71">
+        <v>439401</v>
+      </c>
+      <c r="I71">
+        <v>4914670</v>
+      </c>
+      <c r="J71" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10">
+      <c r="A72" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C72" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D72" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G72" t="s">
+        <v>113</v>
+      </c>
+      <c r="H72">
+        <v>439401</v>
+      </c>
+      <c r="I72">
+        <v>4914670</v>
+      </c>
+      <c r="J72" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" s="9" customFormat="1" ht="15.75" thickBot="1">
+      <c r="A73" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="C73" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="D73" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="F73" s="7" t="s">
+        <v>25</v>
+      </c>
+      <c r="G73" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="H73" s="9">
+        <v>439401</v>
+      </c>
+      <c r="I73" s="9">
+        <v>4914670</v>
+      </c>
+      <c r="J73" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" s="14" customFormat="1">
+      <c r="A74" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C74" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D74" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F74" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="G74" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="H74" s="14">
+        <v>453212</v>
+      </c>
+      <c r="J74" s="16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="75" spans="1:10">
+      <c r="A75" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C75" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D75" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="G75" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="H75">
+        <v>451026</v>
+      </c>
+      <c r="J75" s="16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="76" spans="1:10">
+      <c r="A76" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C76" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D76" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F76" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="G76" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="H76">
+        <v>453140</v>
+      </c>
+      <c r="J76" s="16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="77" spans="1:10">
+      <c r="A77" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C77" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D77" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G77" t="s">
+        <v>120</v>
+      </c>
+      <c r="H77">
+        <v>451117</v>
+      </c>
+      <c r="J77" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="78" spans="1:10">
+      <c r="A78" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C78" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D78" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F78" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G78" t="s">
+        <v>122</v>
+      </c>
+      <c r="H78">
+        <v>451102</v>
+      </c>
+      <c r="J78" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="79" spans="1:10">
+      <c r="A79" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C79" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D79" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="G79" t="s">
+        <v>121</v>
+      </c>
+      <c r="H79">
+        <v>450854</v>
+      </c>
+      <c r="J79" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="80" spans="1:10">
+      <c r="A80" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C80" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D80" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F80" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="G80" t="s">
+        <v>120</v>
+      </c>
+      <c r="H80">
+        <v>427001</v>
+      </c>
+      <c r="J80" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="81" spans="1:10">
+      <c r="A81" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C81" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D81" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G81" t="s">
+        <v>122</v>
+      </c>
+      <c r="H81">
+        <v>426787</v>
+      </c>
+      <c r="J81" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="82" spans="1:10">
+      <c r="A82" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="C82" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D82" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F82" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="G82" t="s">
+        <v>121</v>
+      </c>
+      <c r="H82">
+        <v>426860</v>
+      </c>
+      <c r="J82" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="83" spans="1:10" s="9" customFormat="1" ht="15.75" thickBot="1">
+      <c r="A83" s="7" t="s">
+        <v>116</v>
+      </c>
+      <c r="C83" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="D83" s="13" t="s">
+        <v>8</v>
+      </c>
+      <c r="F83" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="G83" s="9" t="s">
+        <v>124</v>
+      </c>
+      <c r="H83" s="9">
+        <v>435793</v>
+      </c>
+      <c r="J83" s="9" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10">
+      <c r="A84" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C84" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="D84" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F84" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G84" s="16" t="s">
+        <v>127</v>
+      </c>
+      <c r="H84">
+        <v>449455</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10">
+      <c r="A85" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C85" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D85" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F85" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G85" t="s">
+        <v>128</v>
+      </c>
+      <c r="H85">
+        <v>424879</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10">
+      <c r="A86" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C86" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D86" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F86" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G86" t="s">
+        <v>143</v>
+      </c>
+      <c r="H86">
+        <v>449130</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10">
+      <c r="A87" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C87" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D87" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G87" t="s">
+        <v>129</v>
+      </c>
+      <c r="H87">
+        <v>428202</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10">
+      <c r="A88" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C88" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D88" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F88" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G88" t="s">
+        <v>130</v>
+      </c>
+      <c r="H88">
+        <v>445541</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10">
+      <c r="A89" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C89" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="D89" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="F89" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="G89" t="s">
+        <v>131</v>
+      </c>
+      <c r="H89">
+        <v>428519</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10">
+      <c r="A90" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C90" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D90" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F90" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G90" t="s">
+        <v>132</v>
+      </c>
+      <c r="H90">
+        <v>426345</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10">
+      <c r="A91" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C91" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D91" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G91" t="s">
+        <v>133</v>
+      </c>
+      <c r="H91">
+        <v>426771</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10">
+      <c r="A92" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C92" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D92" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F92" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="G92" t="s">
+        <v>134</v>
+      </c>
+      <c r="H92">
+        <v>423324</v>
+      </c>
+    </row>
+    <row r="93" spans="1:10">
+      <c r="A93" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C93" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D93" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="G93" t="s">
+        <v>136</v>
+      </c>
+      <c r="H93">
+        <v>423200</v>
+      </c>
+    </row>
+    <row r="94" spans="1:10">
+      <c r="A94" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C94" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="D94" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F94" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G94" t="s">
+        <v>138</v>
+      </c>
+      <c r="H94">
+        <v>429427</v>
+      </c>
+    </row>
+    <row r="95" spans="1:10">
+      <c r="A95" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C95" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="D95" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F95" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G95" t="s">
+        <v>140</v>
+      </c>
+      <c r="H95">
+        <v>428879</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10">
+      <c r="A96" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="C96" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="D96" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="F96" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="G96" t="s">
+        <v>141</v>
+      </c>
+      <c r="H96">
+        <v>427461</v>
+      </c>
+    </row>
+    <row r="97" spans="6:6">
+      <c r="F97" s="4" t="s">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>